<commit_message>
Updated agents and removed OAuth credentials
</commit_message>
<xml_diff>
--- a/trainer-platform-v8/backend/assets/trainersync_business_register.xlsx
+++ b/trainer-platform-v8/backend/assets/trainersync_business_register.xlsx
@@ -469,7 +469,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20 06:50</t>
+          <t>2026-06-21 05:36</t>
         </is>
       </c>
     </row>
@@ -54516,7 +54516,7 @@
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="32" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="29" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
@@ -56293,7 +56293,7 @@
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>slots_awaiting_confirmation</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr"/>
@@ -56302,7 +56302,7 @@
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Slots Awaiting Confirmation</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Configure Gmail API inbox polling for auto-send
- Added poll_gmail_api_client_inbox() function to fetch emails via Gmail API
- Updated _sync_recent_client_inbox to use Gmail API instead of IMAP
- No need for IMAP credentials anymore - uses existing Gmail OAuth token
- System now receives, processes, and auto-replies to client emails
- Support for IMAP will be added in production when configured
</commit_message>
<xml_diff>
--- a/trainer-platform-v8/backend/assets/trainersync_business_register.xlsx
+++ b/trainer-platform-v8/backend/assets/trainersync_business_register.xlsx
@@ -469,7 +469,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23 05:13</t>
+          <t>2026-06-23 06:58</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>66</t>
         </is>
       </c>
     </row>
@@ -7782,7 +7782,7 @@
       <c r="L135" s="2" t="inlineStr"/>
       <c r="M135" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N135" s="2" t="inlineStr">
@@ -8392,7 +8392,7 @@
       <c r="L145" s="2" t="inlineStr"/>
       <c r="M145" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N145" s="2" t="inlineStr">
@@ -8819,7 +8819,7 @@
       <c r="L152" s="2" t="inlineStr"/>
       <c r="M152" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N152" s="2" t="inlineStr">
@@ -9063,12 +9063,12 @@
       <c r="L156" s="2" t="inlineStr"/>
       <c r="M156" s="2" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N156" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="O156" s="2" t="inlineStr">
@@ -49037,7 +49037,7 @@
       <c r="L941" s="2" t="inlineStr"/>
       <c r="M941" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N941" s="2" t="inlineStr">
@@ -49094,7 +49094,7 @@
       <c r="L942" s="2" t="inlineStr"/>
       <c r="M942" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N942" s="2" t="inlineStr">
@@ -49375,7 +49375,7 @@
       <c r="L947" s="2" t="inlineStr"/>
       <c r="M947" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N947" s="2" t="inlineStr">
@@ -49970,7 +49970,7 @@
       <c r="L958" s="2" t="inlineStr"/>
       <c r="M958" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N958" s="2" t="inlineStr">
@@ -50642,12 +50642,12 @@
       <c r="L970" s="2" t="inlineStr"/>
       <c r="M970" s="2" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N970" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="O970" s="2" t="inlineStr">
@@ -50813,12 +50813,12 @@
       <c r="L973" s="2" t="inlineStr"/>
       <c r="M973" s="2" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N973" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="O973" s="2" t="inlineStr">
@@ -50976,7 +50976,7 @@
       <c r="L976" s="2" t="inlineStr"/>
       <c r="M976" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N976" s="2" t="inlineStr">
@@ -51383,7 +51383,7 @@
       <c r="L983" s="2" t="inlineStr"/>
       <c r="M983" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N983" s="2" t="inlineStr">
@@ -51497,12 +51497,12 @@
       <c r="L985" s="2" t="inlineStr"/>
       <c r="M985" s="2" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N985" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="O985" s="2" t="inlineStr">
@@ -51847,7 +51847,7 @@
       <c r="L991" s="2" t="inlineStr"/>
       <c r="M991" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N991" s="2" t="inlineStr">
@@ -52071,7 +52071,7 @@
       <c r="L995" s="2" t="inlineStr"/>
       <c r="M995" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N995" s="2" t="inlineStr">
@@ -52755,7 +52755,7 @@
       <c r="L1007" s="2" t="inlineStr"/>
       <c r="M1007" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N1007" s="2" t="inlineStr">
@@ -53154,7 +53154,7 @@
       <c r="L1014" s="2" t="inlineStr"/>
       <c r="M1014" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N1014" s="2" t="inlineStr">
@@ -53386,7 +53386,7 @@
       <c r="L1018" s="2" t="inlineStr"/>
       <c r="M1018" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N1018" s="2" t="inlineStr">
@@ -53447,7 +53447,7 @@
       <c r="L1019" s="2" t="inlineStr"/>
       <c r="M1019" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N1019" s="2" t="inlineStr">
@@ -53508,7 +53508,7 @@
       <c r="L1020" s="2" t="inlineStr"/>
       <c r="M1020" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N1020" s="2" t="inlineStr">
@@ -53626,7 +53626,7 @@
       <c r="L1022" s="2" t="inlineStr"/>
       <c r="M1022" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N1022" s="2" t="inlineStr">
@@ -53858,12 +53858,12 @@
       <c r="L1026" s="2" t="inlineStr"/>
       <c r="M1026" s="2" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N1026" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="O1026" s="2" t="inlineStr">
@@ -54090,12 +54090,12 @@
       <c r="L1030" s="2" t="inlineStr"/>
       <c r="M1030" s="2" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N1030" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="O1030" s="2" t="inlineStr">
@@ -54253,12 +54253,12 @@
       <c r="L1033" s="2" t="inlineStr"/>
       <c r="M1033" s="2" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N1033" s="2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="O1033" s="2" t="inlineStr">
@@ -54503,7 +54503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q58"/>
+  <dimension ref="A1:Q67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -54620,36 +54620,28 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>REQ-F7179BE8</t>
+          <t>REQ-5D30BAFA</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Sujitha</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>info@kodnest.com</t>
+          <t>sujithaofficial784@gmail.com</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>IT industry, placement-focused training</t>
+          <t>DevOps</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>22nd June 2026</t>
-        </is>
-      </c>
+      <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>online and offline hybrid</t>
-        </is>
-      </c>
+      <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -54667,7 +54659,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20 06:18</t>
+          <t>2026-06-23 06:36</t>
         </is>
       </c>
     </row>
@@ -54679,40 +54671,32 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>REQ-E6FA1D86</t>
+          <t>REQ-0D10D857</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Muttarasu Sujitha</t>
+          <t>Saeed Ahmed Davawala</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>sujithamuttarasu@gmail.com</t>
+          <t>saeedd77@gmail.com</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Full Stack</t>
+          <t>Calendly</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Next Monday</t>
-        </is>
-      </c>
+      <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>online</t>
-        </is>
-      </c>
+      <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>active</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr"/>
@@ -54721,12 +54705,12 @@
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 11:51</t>
+          <t>2026-06-23 06:19</t>
         </is>
       </c>
     </row>
@@ -54738,38 +54722,38 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>REQ-C0B7D403</t>
+          <t>REQ-16F2A5DA</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Suman Nandy</t>
+          <t>null</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>nandy.suman90@gmail.com</t>
+          <t>naukrialerts@naukri.com</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Python, Agentic AI Trainer</t>
+          <t>Salesforce</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>21st June, 2026</t>
+          <t>null</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>8 Hours</t>
+          <t>null</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>null</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
@@ -54789,7 +54773,7 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 11:48</t>
+          <t>2026-06-23 06:02</t>
         </is>
       </c>
     </row>
@@ -54801,22 +54785,22 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>REQ-A47C978B</t>
+          <t>REQ-56627709</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Muttarasu Sujitha</t>
+          <t>Ahmed</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>sujithamuttarasu@gmail.com</t>
+          <t>trainer.oracledb@gmail.com</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Full Stack Trainer Requirement</t>
+          <t>Oracle DB Administration</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
@@ -54826,7 +54810,7 @@
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>active</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr"/>
@@ -54835,12 +54819,12 @@
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 11:46</t>
+          <t>2026-06-23 05:55</t>
         </is>
       </c>
     </row>
@@ -54852,36 +54836,32 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>REQ-8EE65AB4</t>
+          <t>REQ-CC3A15B6</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>muttarasusujitha</t>
+          <t>Ashok IT</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>reply+bft4frcf4mrcfrhidvzo2ftkvyhb3evbnhhqaaaaaemaied5@reply.github.com</t>
+          <t>info@ashokit.in</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>natural-language trainer requirement</t>
+          <t>Generative AI, Spring Boot, Ollama</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>next week</t>
+          <t>21 June</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
+      <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr">
         <is>
@@ -54899,7 +54879,7 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 11:45</t>
+          <t>2026-06-23 05:41</t>
         </is>
       </c>
     </row>
@@ -54911,28 +54891,36 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>REQ-720B49B3</t>
+          <t>REQ-DE803627</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Sujitha</t>
+          <t>KodNest Team</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>sujithaofficial784@gmail.com</t>
+          <t>info@kodnest.com</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Full Stack Trainer Requirement</t>
+          <t>IT industry, online &amp; offline</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>22nd June 2026</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>online &amp; offline</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr">
         <is>
@@ -54950,7 +54938,7 @@
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 11:43</t>
+          <t>2026-06-23 05:40</t>
         </is>
       </c>
     </row>
@@ -54962,26 +54950,30 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>REQ-FC3384AB</t>
+          <t>REQ-24E171E2</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Sujitha</t>
+          <t>Suman Nandy</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>sujithaofficial784@gmail.com</t>
+          <t>nandy.suman90@gmail.com</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Full Stack Training</t>
+          <t>DevOps</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Next Monday</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr"/>
@@ -55001,7 +54993,7 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 11:42</t>
+          <t>2026-06-23 05:40</t>
         </is>
       </c>
     </row>
@@ -55013,38 +55005,34 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>REQ-9BD53F43</t>
+          <t>REQ-AF7A6838</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Sujitha</t>
+          <t>Suman Nandy</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>sujithaofficial784@gmail.com</t>
+          <t>nandy.suman90@gmail.com</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Full Stack</t>
+          <t>null</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>22nd June 2026 onwards</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>7:00 PM – 9:00 PM IST</t>
-        </is>
-      </c>
+          <t>25/06/2026</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>null</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
@@ -55064,7 +55052,7 @@
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 11:40</t>
+          <t>2026-06-23 05:39</t>
         </is>
       </c>
     </row>
@@ -55076,32 +55064,28 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>REQ-6C9EE1D8</t>
+          <t>REQ-CEFB8A8E</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Isa Bell</t>
+          <t>Sujitha</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>isa.bell@twilio.com</t>
+          <t>sujithaofficial585@gmail.com</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>custom build with Twilio APIs or connecting Twilio into a platform they already use or ready-made partner solution</t>
+          <t>Oracle DBA</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>hybrid</t>
-        </is>
-      </c>
+      <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -55119,7 +55103,7 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 11:39</t>
+          <t>2026-06-23 05:37</t>
         </is>
       </c>
     </row>
@@ -55131,38 +55115,34 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>REQ-51D6D412</t>
+          <t>REQ-F7179BE8</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Sujitha</t>
+          <t>null</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>sujithaofficial784@gmail.com</t>
+          <t>info@kodnest.com</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Full Stack Development</t>
+          <t>IT industry, placement-focused training</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>01/07/2026 to 20/07/2026</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>9:00 AM to 4:00 PM</t>
-        </is>
-      </c>
+          <t>22nd June 2026</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Classroom</t>
+          <t>online and offline hybrid</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr"/>
@@ -55182,7 +55162,7 @@
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 11:38</t>
+          <t>2026-06-20 06:18</t>
         </is>
       </c>
     </row>
@@ -55194,7 +55174,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>REQ-AE3DF43B</t>
+          <t>REQ-E6FA1D86</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -55213,11 +55193,15 @@
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Next Monday</t>
+        </is>
+      </c>
       <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>hybrid</t>
+          <t>online</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr"/>
@@ -55237,7 +55221,7 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 11:37</t>
+          <t>2026-06-19 11:51</t>
         </is>
       </c>
     </row>
@@ -55249,34 +55233,38 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>REQ-7EE2C1C9</t>
+          <t>REQ-C0B7D403</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Stratemis HR Technologies</t>
+          <t>Suman Nandy</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>careerservices@career247.com</t>
+          <t>nandy.suman90@gmail.com</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>HR Basics, Excel, Communication</t>
+          <t>Python, Agentic AI Trainer</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>6 Months</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr"/>
+          <t>21st June, 2026</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>8 Hours</t>
+        </is>
+      </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>hybrid</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr"/>
@@ -55296,7 +55284,7 @@
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 11:36</t>
+          <t>2026-06-19 11:48</t>
         </is>
       </c>
     </row>
@@ -55308,40 +55296,32 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>REQ-FA303118</t>
+          <t>REQ-A47C978B</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Sujitha</t>
+          <t>Muttarasu Sujitha</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>sujithaofficial784@gmail.com</t>
+          <t>sujithamuttarasu@gmail.com</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Professional Training Program</t>
+          <t>Full Stack Trainer Requirement</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>9 AM to 4 PM</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>online/offline (as applicable)</t>
-        </is>
-      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr"/>
@@ -55350,12 +55330,12 @@
       <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 11:35</t>
+          <t>2026-06-19 11:46</t>
         </is>
       </c>
     </row>
@@ -55367,22 +55347,22 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>REQ-10114C4B</t>
+          <t>REQ-8EE65AB4</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Sujitha</t>
+          <t>muttarasusujitha</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>sujithaofficial784@gmail.com</t>
+          <t>reply+bft4frcf4mrcfrhidvzo2ftkvyhb3evbnhhqaaaaaemaied5@reply.github.com</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>training program, skills required not specified</t>
+          <t>natural-language trainer requirement</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr"/>
@@ -55391,14 +55371,10 @@
           <t>next week</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>9 AM to 4 PM</t>
-        </is>
-      </c>
+      <c r="H15" s="2" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>online</t>
+          <t>null</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr"/>
@@ -55418,7 +55394,7 @@
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 11:34</t>
+          <t>2026-06-19 11:45</t>
         </is>
       </c>
     </row>
@@ -55430,40 +55406,28 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>REQ-BF6489AA</t>
+          <t>REQ-720B49B3</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Sujitha</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>info@kodnest.com</t>
+          <t>sujithaofficial784@gmail.com</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Full Stack Development or Software Testing</t>
+          <t>Full Stack Trainer Requirement</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>18th May 2026</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>online &amp; offline</t>
-        </is>
-      </c>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr">
         <is>
@@ -55481,7 +55445,7 @@
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 11:32</t>
+          <t>2026-06-19 11:43</t>
         </is>
       </c>
     </row>
@@ -55493,36 +55457,28 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>REQ-645D4064</t>
+          <t>REQ-FC3384AB</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Sujitha</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>info@kodnest.com</t>
+          <t>sujithaofficial784@gmail.com</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Full Stack Development or Software Testing</t>
+          <t>Full Stack Training</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>20th April 2026</t>
-        </is>
-      </c>
+      <c r="G17" s="2" t="inlineStr"/>
       <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>Online &amp; Offline</t>
-        </is>
-      </c>
+      <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr">
         <is>
@@ -55540,7 +55496,7 @@
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 11:29</t>
+          <t>2026-06-19 11:42</t>
         </is>
       </c>
     </row>
@@ -55552,34 +55508,38 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>REQ-C2D2EB31</t>
+          <t>REQ-9BD53F43</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Sujitha</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>info@kodnest.com</t>
+          <t>sujithaofficial784@gmail.com</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Full Stack Development &amp; Testing</t>
+          <t>Full Stack</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>30th March 2026</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr"/>
+          <t>22nd June 2026 onwards</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>7:00 PM – 9:00 PM IST</t>
+        </is>
+      </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>hybrid</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
@@ -55599,7 +55559,7 @@
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 11:28</t>
+          <t>2026-06-19 11:40</t>
         </is>
       </c>
     </row>
@@ -55611,28 +55571,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>REQ-987472B5</t>
+          <t>REQ-6C9EE1D8</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Saeed Ahmed Davawala</t>
+          <t>Isa Bell</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>saeedd77@gmail.com</t>
+          <t>isa.bell@twilio.com</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>custom build with Twilio APIs or connecting Twilio into a platform they already use or ready-made partner solution</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr">
         <is>
@@ -55650,7 +55614,7 @@
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 11:02</t>
+          <t>2026-06-19 11:39</t>
         </is>
       </c>
     </row>
@@ -55662,34 +55626,38 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>REQ-9CADDFEE</t>
+          <t>REQ-51D6D412</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Sujitha</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>vinila@code.iitm.ac.in</t>
+          <t>sujithaofficial784@gmail.com</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning</t>
+          <t>Full Stack Development</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>August 22, 2025</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr"/>
+          <t>01/07/2026 to 20/07/2026</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>9:00 AM to 4:00 PM</t>
+        </is>
+      </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>hybrid</t>
+          <t>Classroom</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr"/>
@@ -55709,7 +55677,7 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 10:56</t>
+          <t>2026-06-19 11:38</t>
         </is>
       </c>
     </row>
@@ -55721,44 +55689,36 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>REQ-9A0B3580</t>
+          <t>REQ-AE3DF43B</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Swetha Kothapalli</t>
+          <t>Muttarasu Sujitha</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>swetha.kothapalli@innomatics.in</t>
+          <t>sujithamuttarasu@gmail.com</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Data Analysis with Python</t>
+          <t>Full Stack</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>Monday, 28th July 2025</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>6:00 PM to 7:30 PM</t>
-        </is>
-      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>online</t>
+          <t>hybrid</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr"/>
@@ -55767,12 +55727,12 @@
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 10:55</t>
+          <t>2026-06-19 11:37</t>
         </is>
       </c>
     </row>
@@ -55784,38 +55744,34 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>REQ-2FF53168</t>
+          <t>REQ-7EE2C1C9</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Muttarasu Sujitha</t>
+          <t>Stratemis HR Technologies</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>certificate@pantechelearning.com</t>
+          <t>careerservices@career247.com</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Generative Artificial Intelligence</t>
+          <t>HR Basics, Excel, Communication</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>1st FEB - 2nd FEB 2025</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>6:30 pm - 8:30 pm</t>
-        </is>
-      </c>
+          <t>6 Months</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>online</t>
+          <t>hybrid</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr"/>
@@ -55835,7 +55791,7 @@
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 10:37</t>
+          <t>2026-06-19 11:36</t>
         </is>
       </c>
     </row>
@@ -55847,38 +55803,34 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>REQ-CB38A055</t>
+          <t>REQ-FA303118</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>MUTTARASU SUJITHA</t>
+          <t>Sujitha</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>certificate@pantechelearning.com</t>
+          <t>sujithaofficial784@gmail.com</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Generative AI</t>
+          <t>Professional Training Program</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>1st FEB - 2nd FEB 2025</t>
-        </is>
-      </c>
+      <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>6:30 pm - 8:30 pm</t>
+          <t>9 AM to 4 PM</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>online</t>
+          <t>online/offline (as applicable)</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr"/>
@@ -55898,7 +55850,7 @@
       </c>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 10:36</t>
+          <t>2026-06-19 11:35</t>
         </is>
       </c>
     </row>
@@ -55910,28 +55862,40 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>REQ-EBD8399B</t>
+          <t>REQ-10114C4B</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Muttarasu Sujitha</t>
+          <t>Sujitha</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>sujithamuttarasu@gmail.com</t>
+          <t>sujithaofficial784@gmail.com</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>DevOps</t>
+          <t>training program, skills required not specified</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>next week</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>9 AM to 4 PM</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr">
         <is>
@@ -55949,7 +55913,7 @@
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 10:35</t>
+          <t>2026-06-19 11:34</t>
         </is>
       </c>
     </row>
@@ -55961,7 +55925,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>REQ-9D1422CB</t>
+          <t>REQ-BF6489AA</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -55971,28 +55935,28 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>certificate@pantechelearning.com</t>
+          <t>info@kodnest.com</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Advanced Analytics With Power BI</t>
+          <t>Full Stack Development or Software Testing</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>6.12.2024 - 7.12.2024</t>
+          <t>18th May 2026</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>5:30 to 7:30 PM</t>
+          <t>null</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>online</t>
+          <t>online &amp; offline</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr"/>
@@ -56012,7 +55976,7 @@
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 10:32</t>
+          <t>2026-06-19 11:32</t>
         </is>
       </c>
     </row>
@@ -56024,30 +55988,34 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>REQ-7198BEBA</t>
+          <t>REQ-645D4064</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Muttarasu Sujitha</t>
+          <t>null</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>certificate@pantechelearning.com</t>
+          <t>info@kodnest.com</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Artificial Intelligence, Machine Learning &amp; Deep Learning, Generative AI &amp; Natural Language Processing (NLP), Data Science &amp; Data Analytics</t>
+          <t>Full Stack Development or Software Testing</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>20th April 2026</t>
+        </is>
+      </c>
       <c r="H26" s="2" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>hybrid</t>
+          <t>Online &amp; Offline</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr"/>
@@ -56067,7 +56035,7 @@
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 10:31</t>
+          <t>2026-06-19 11:29</t>
         </is>
       </c>
     </row>
@@ -56079,7 +56047,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>REQ-95F7F349</t>
+          <t>REQ-C2D2EB31</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -56089,28 +56057,24 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>certificate@pantechelearning.com</t>
+          <t>info@kodnest.com</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Machine learning with Data Analytics</t>
+          <t>Full Stack Development &amp; Testing</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>27-11-2024 &amp; 28-11-2024</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>5:00 pm - 7:00 pm</t>
-        </is>
-      </c>
+          <t>30th March 2026</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr"/>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>online</t>
+          <t>hybrid</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr"/>
@@ -56130,7 +56094,7 @@
       </c>
       <c r="Q27" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 10:30</t>
+          <t>2026-06-19 11:28</t>
         </is>
       </c>
     </row>
@@ -56142,40 +56106,28 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>REQ-430CB350</t>
+          <t>REQ-987472B5</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Saeed Ahmed Davawala</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>certificate@pantechelearning.com</t>
+          <t>saeedd77@gmail.com</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Machine learning with Data Analytics</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>26-11-2024 &amp; 27-11-2024</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>5:00 pm - 7:00 pm</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>online</t>
-        </is>
-      </c>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr">
         <is>
@@ -56193,7 +56145,7 @@
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 10:29</t>
+          <t>2026-06-19 11:02</t>
         </is>
       </c>
     </row>
@@ -56205,30 +56157,34 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>REQ-12961278</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr"/>
+          <t>REQ-9CADDFEE</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>onlinecourses@nptel.iitm.ac.in</t>
+          <t>vinila@code.iitm.ac.in</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Programming in Java</t>
+          <t>Machine Learning</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Week-07</t>
+          <t>August 22, 2025</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>online</t>
+          <t>hybrid</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
@@ -56248,7 +56204,7 @@
       </c>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 10:25</t>
+          <t>2026-06-19 10:56</t>
         </is>
       </c>
     </row>
@@ -56260,40 +56216,44 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>REQ-482B0DCF</t>
+          <t>REQ-9A0B3580</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Sujitha</t>
+          <t>Swetha Kothapalli</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>sujithaofficial784@gmail.com</t>
+          <t>swetha.kothapalli@innomatics.in</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>DevOps</t>
+          <t>Data Analysis with Python</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2nd Week of July 2026</t>
+          <t>Monday, 28th July 2025</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>10:00 AM – 1:00 PM IST</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr"/>
+          <t>6:00 PM to 7:30 PM</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>slots_awaiting_confirmation</t>
+          <t>active</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr"/>
@@ -56302,12 +56262,12 @@
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>Slots Awaiting Confirmation</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 10:24</t>
+          <t>2026-06-19 10:55</t>
         </is>
       </c>
     </row>
@@ -56319,27 +56279,35 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>REQ-7BCEF2C9</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr"/>
+          <t>REQ-2FF53168</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Muttarasu Sujitha</t>
+        </is>
+      </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>onlinecourses@nptel.iitm.ac.in</t>
+          <t>certificate@pantechelearning.com</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Programming in Java</t>
+          <t>Generative Artificial Intelligence</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr"/>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Week-05</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr"/>
+          <t>1st FEB - 2nd FEB 2025</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>6:30 pm - 8:30 pm</t>
+        </is>
+      </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
           <t>online</t>
@@ -56362,7 +56330,7 @@
       </c>
       <c r="Q31" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 10:24</t>
+          <t>2026-06-19 10:37</t>
         </is>
       </c>
     </row>
@@ -56374,27 +56342,35 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>REQ-DB2C36BE</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr"/>
+          <t>REQ-CB38A055</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>MUTTARASU SUJITHA</t>
+        </is>
+      </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>onlinecourses@nptel.iitm.ac.in</t>
+          <t>certificate@pantechelearning.com</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Programming in Java</t>
+          <t>Generative AI</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Week-03</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr"/>
+          <t>1st FEB - 2nd FEB 2025</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>6:30 pm - 8:30 pm</t>
+        </is>
+      </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
           <t>online</t>
@@ -56417,7 +56393,7 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 10:23</t>
+          <t>2026-06-19 10:36</t>
         </is>
       </c>
     </row>
@@ -56429,17 +56405,17 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>REQ-11E949B6</t>
+          <t>REQ-EBD8399B</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Ravi Rakesh</t>
+          <t>Muttarasu Sujitha</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>rthi2009@gmail.com</t>
+          <t>sujithamuttarasu@gmail.com</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -56450,11 +56426,7 @@
       <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="2" t="inlineStr"/>
       <c r="H33" s="2" t="inlineStr"/>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>online</t>
-        </is>
-      </c>
+      <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="inlineStr"/>
       <c r="K33" s="2" t="inlineStr">
         <is>
@@ -56472,7 +56444,7 @@
       </c>
       <c r="Q33" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 10:11</t>
+          <t>2026-06-19 10:35</t>
         </is>
       </c>
     </row>
@@ -56484,28 +56456,40 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>REQ-950651BA</t>
+          <t>REQ-9D1422CB</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Ravi Rakesh</t>
+          <t>null</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>rthi2009@gmail.com</t>
+          <t>certificate@pantechelearning.com</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Python, Agentic AI</t>
+          <t>Advanced Analytics With Power BI</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>6.12.2024 - 7.12.2024</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>5:30 to 7:30 PM</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
       <c r="J34" s="2" t="inlineStr"/>
       <c r="K34" s="2" t="inlineStr">
         <is>
@@ -56523,7 +56507,7 @@
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18 07:24</t>
+          <t>2026-06-19 10:32</t>
         </is>
       </c>
     </row>
@@ -56535,38 +56519,30 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>REQ-7CDED142</t>
+          <t>REQ-7198BEBA</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Suman Nandy</t>
+          <t>Muttarasu Sujitha</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>nandy.suman90@gmail.com</t>
+          <t>certificate@pantechelearning.com</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Python, Agentic AI</t>
+          <t>Artificial Intelligence, Machine Learning &amp; Deep Learning, Generative AI &amp; Natural Language Processing (NLP), Data Science &amp; Data Analytics</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>21st June, 2026</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>8 Hours</t>
-        </is>
-      </c>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr"/>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>hybrid</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr"/>
@@ -56586,7 +56562,7 @@
       </c>
       <c r="Q35" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18 07:14</t>
+          <t>2026-06-19 10:31</t>
         </is>
       </c>
     </row>
@@ -56598,28 +56574,40 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>REQ-488233F4</t>
+          <t>REQ-95F7F349</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Sujitha</t>
+          <t>null</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>sujithaofficial784@gmail.com</t>
+          <t>certificate@pantechelearning.com</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>DevOps</t>
+          <t>Machine learning with Data Analytics</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="inlineStr"/>
-      <c r="I36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>27-11-2024 &amp; 28-11-2024</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>5:00 pm - 7:00 pm</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
       <c r="J36" s="2" t="inlineStr"/>
       <c r="K36" s="2" t="inlineStr">
         <is>
@@ -56637,7 +56625,7 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18 07:04</t>
+          <t>2026-06-19 10:30</t>
         </is>
       </c>
     </row>
@@ -56649,28 +56637,40 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>REQ-D02518CB</t>
+          <t>REQ-430CB350</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Suman Nandy</t>
+          <t>null</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>nandy.suman90@gmail.com</t>
+          <t>certificate@pantechelearning.com</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Python, Agentic AI</t>
+          <t>Machine learning with Data Analytics</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr"/>
-      <c r="G37" s="2" t="inlineStr"/>
-      <c r="H37" s="2" t="inlineStr"/>
-      <c r="I37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>26-11-2024 &amp; 27-11-2024</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>5:00 pm - 7:00 pm</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
       <c r="J37" s="2" t="inlineStr"/>
       <c r="K37" s="2" t="inlineStr">
         <is>
@@ -56688,7 +56688,7 @@
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18 06:34</t>
+          <t>2026-06-19 10:29</t>
         </is>
       </c>
     </row>
@@ -56700,32 +56700,32 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>REQ-93EA4DAA</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>Ashok IT</t>
-        </is>
-      </c>
+          <t>REQ-12961278</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr"/>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>info@ashokit.in</t>
+          <t>onlinecourses@nptel.iitm.ac.in</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>Programming in Java</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr"/>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>13 June</t>
+          <t>Week-07</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
-      <c r="I38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
       <c r="J38" s="2" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr">
         <is>
@@ -56743,7 +56743,7 @@
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18 04:54</t>
+          <t>2026-06-19 10:25</t>
         </is>
       </c>
     </row>
@@ -56755,32 +56755,40 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>REQ-4C16F195</t>
+          <t>REQ-482B0DCF</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Ashok</t>
+          <t>Sujitha</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>info@ashokit.in</t>
+          <t>sujithaofficial784@gmail.com</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>DevOps</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr"/>
-      <c r="G39" s="2" t="inlineStr"/>
-      <c r="H39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>2nd Week of July 2026</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>10:00 AM – 1:00 PM IST</t>
+        </is>
+      </c>
       <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="2" t="inlineStr"/>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>slots_awaiting_confirmation</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr"/>
@@ -56789,12 +56797,12 @@
       <c r="O39" s="2" t="inlineStr"/>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Slots Awaiting Confirmation</t>
         </is>
       </c>
       <c r="Q39" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18 04:53</t>
+          <t>2026-06-19 10:24</t>
         </is>
       </c>
     </row>
@@ -56806,32 +56814,32 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>REQ-4B3C3D54</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Ashok</t>
-        </is>
-      </c>
+          <t>REQ-7BCEF2C9</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr"/>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>info@ashokit.in</t>
+          <t>onlinecourses@nptel.iitm.ac.in</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Bash Shell Scripting</t>
+          <t>Programming in Java</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Today at 08:00 PM</t>
+          <t>Week-05</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
-      <c r="I40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
       <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr">
         <is>
@@ -56849,7 +56857,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18 04:51</t>
+          <t>2026-06-19 10:24</t>
         </is>
       </c>
     </row>
@@ -56861,28 +56869,32 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>REQ-96F777A0</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Ashok IT</t>
-        </is>
-      </c>
+          <t>REQ-DB2C36BE</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr"/>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>info@ashokit.in</t>
+          <t>onlinecourses@nptel.iitm.ac.in</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Python, Agentic AI</t>
+          <t>Programming in Java</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr"/>
-      <c r="G41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Week-03</t>
+        </is>
+      </c>
       <c r="H41" s="2" t="inlineStr"/>
-      <c r="I41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
       <c r="J41" s="2" t="inlineStr"/>
       <c r="K41" s="2" t="inlineStr">
         <is>
@@ -56900,7 +56912,7 @@
       </c>
       <c r="Q41" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18 04:49</t>
+          <t>2026-06-19 10:23</t>
         </is>
       </c>
     </row>
@@ -56912,28 +56924,32 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>REQ-D068F9F5</t>
+          <t>REQ-11E949B6</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Ashok IT</t>
+          <t>Ravi Rakesh</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>info@ashokit.in</t>
+          <t>rthi2009@gmail.com</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>DevOps</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr"/>
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
       <c r="J42" s="2" t="inlineStr"/>
       <c r="K42" s="2" t="inlineStr">
         <is>
@@ -56951,7 +56967,7 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18 04:46</t>
+          <t>2026-06-19 10:11</t>
         </is>
       </c>
     </row>
@@ -56963,36 +56979,28 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>REQ-C57E228B</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr"/>
+          <t>REQ-950651BA</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Ravi Rakesh</t>
+        </is>
+      </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>info@ashokit.in</t>
+          <t>rthi2009@gmail.com</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>.NET Core Microservices</t>
+          <t>Python, Agentic AI</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr"/>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>next week</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>9 AM to 4 PM</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t>online</t>
-        </is>
-      </c>
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr"/>
       <c r="J43" s="2" t="inlineStr"/>
       <c r="K43" s="2" t="inlineStr">
         <is>
@@ -57010,7 +57018,7 @@
       </c>
       <c r="Q43" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11 11:49</t>
+          <t>2026-06-18 07:24</t>
         </is>
       </c>
     </row>
@@ -57022,28 +57030,40 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>REQ-E8AD8FDD</t>
+          <t>REQ-7CDED142</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Calhan Technologies</t>
+          <t>Suman Nandy</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>vikasb.consult@gmail.com</t>
+          <t>nandy.suman90@gmail.com</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>GCP Cloud</t>
+          <t>Python, Agentic AI</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" s="2" t="inlineStr"/>
-      <c r="H44" s="2" t="inlineStr"/>
-      <c r="I44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>21st June, 2026</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>8 Hours</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
       <c r="J44" s="2" t="inlineStr"/>
       <c r="K44" s="2" t="inlineStr">
         <is>
@@ -57061,7 +57081,7 @@
       </c>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11 11:20</t>
+          <t>2026-06-18 07:14</t>
         </is>
       </c>
     </row>
@@ -57073,22 +57093,22 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>REQ-379FAF6E</t>
+          <t>REQ-488233F4</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Suman Nandy</t>
+          <t>Sujitha</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>nandy.suman90@gmail.com</t>
+          <t>sujithaofficial784@gmail.com</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>PostgreSQL</t>
+          <t>DevOps</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr"/>
@@ -57112,7 +57132,7 @@
       </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11 03:54</t>
+          <t>2026-06-18 07:04</t>
         </is>
       </c>
     </row>
@@ -57124,54 +57144,46 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>REQ-A6E19094</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr"/>
+          <t>REQ-D02518CB</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Suman Nandy</t>
+        </is>
+      </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>info@ashokit.in</t>
+          <t>nandy.suman90@gmail.com</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>GCP Cloud</t>
+          <t>Python, Agentic AI</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr"/>
       <c r="G46" s="2" t="inlineStr"/>
       <c r="H46" s="2" t="inlineStr"/>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>online</t>
-        </is>
-      </c>
+      <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>selected</t>
-        </is>
-      </c>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>Vikas Kumar B.</t>
-        </is>
-      </c>
-      <c r="M46" s="2" t="inlineStr">
-        <is>
-          <t>TR-6C67624B</t>
-        </is>
-      </c>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr"/>
+      <c r="M46" s="2" t="inlineStr"/>
       <c r="N46" s="2" t="inlineStr"/>
       <c r="O46" s="2" t="inlineStr"/>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>Selected / active requirement</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="Q46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10 10:16</t>
+          <t>2026-06-18 06:34</t>
         </is>
       </c>
     </row>
@@ -57183,17 +57195,17 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>REQ-793B9BF0</t>
+          <t>REQ-93EA4DAA</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Saeed Ahmed Davawala</t>
+          <t>Ashok IT</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>saeedd77@gmail.com</t>
+          <t>info@ashokit.in</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -57202,7 +57214,11 @@
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr"/>
-      <c r="G47" s="2" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>13 June</t>
+        </is>
+      </c>
       <c r="H47" s="2" t="inlineStr"/>
       <c r="I47" s="2" t="inlineStr"/>
       <c r="J47" s="2" t="inlineStr"/>
@@ -57222,7 +57238,7 @@
       </c>
       <c r="Q47" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10 03:58</t>
+          <t>2026-06-18 04:54</t>
         </is>
       </c>
     </row>
@@ -57234,22 +57250,22 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>REQ-8397589F</t>
+          <t>REQ-4C16F195</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Ahmed</t>
+          <t>Ashok</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>trainer.oracledb@gmail.com</t>
+          <t>info@ashokit.in</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>OEM Technology Programs</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr"/>
@@ -57273,7 +57289,7 @@
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10 03:58</t>
+          <t>2026-06-18 04:53</t>
         </is>
       </c>
     </row>
@@ -57285,12 +57301,12 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>REQ-8F5B6993</t>
+          <t>REQ-4B3C3D54</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Ashok IT</t>
+          <t>Ashok</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -57300,17 +57316,21 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>Bash Shell Scripting</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr"/>
-      <c r="G49" s="2" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Today at 08:00 PM</t>
+        </is>
+      </c>
       <c r="H49" s="2" t="inlineStr"/>
       <c r="I49" s="2" t="inlineStr"/>
       <c r="J49" s="2" t="inlineStr"/>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>closed</t>
+          <t>active</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr"/>
@@ -57319,12 +57339,12 @@
       <c r="O49" s="2" t="inlineStr"/>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="Q49" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09 10:00</t>
+          <t>2026-06-18 04:51</t>
         </is>
       </c>
     </row>
@@ -57336,32 +57356,28 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>REQ-060645F0</t>
+          <t>REQ-96F777A0</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Manoj Nair</t>
+          <t>Ashok IT</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>manojanair1@yahoo.com</t>
+          <t>info@ashokit.in</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Contract Law Essentials, Contract Drafting &amp; Negotiation, Legal Risk Management, Strategic Legal Leadership</t>
+          <t>Python, Agentic AI</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr"/>
       <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr"/>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>hybrid</t>
-        </is>
-      </c>
+      <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" s="2" t="inlineStr">
         <is>
@@ -57379,7 +57395,7 @@
       </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09 09:13</t>
+          <t>2026-06-18 04:49</t>
         </is>
       </c>
     </row>
@@ -57391,22 +57407,22 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>REQ-66017F20</t>
+          <t>REQ-D068F9F5</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Preeti Saxena</t>
+          <t>Ashok IT</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>preeti.saxena@pynetlabs.com</t>
+          <t>info@ashokit.in</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>OEM Technology Programs</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr"/>
@@ -57430,7 +57446,7 @@
       </c>
       <c r="Q51" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09 09:12</t>
+          <t>2026-06-18 04:46</t>
         </is>
       </c>
     </row>
@@ -57442,34 +57458,34 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>REQ-DB584D6B</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Sushmita Mukherjee Ganguly</t>
-        </is>
-      </c>
+          <t>REQ-C57E228B</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr"/>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>sushmita@agsuitetech.com</t>
+          <t>info@ashokit.in</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Oracle Netsuite</t>
+          <t>.NET Core Microservices</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr"/>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>null</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr"/>
+          <t>next week</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>9 AM to 4 PM</t>
+        </is>
+      </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>online</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr"/>
@@ -57489,7 +57505,7 @@
       </c>
       <c r="Q52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09 09:12</t>
+          <t>2026-06-11 11:49</t>
         </is>
       </c>
     </row>
@@ -57501,22 +57517,22 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>REQ-6C6E9EEE</t>
+          <t>REQ-E8AD8FDD</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Sushmita Mukherjee Ganguly</t>
+          <t>Calhan Technologies</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>sushmita@agsuitetech.com</t>
+          <t>vikasb.consult@gmail.com</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Oracle Netsuite</t>
+          <t>GCP Cloud</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr"/>
@@ -57540,7 +57556,7 @@
       </c>
       <c r="Q53" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09 09:11</t>
+          <t>2026-06-11 11:20</t>
         </is>
       </c>
     </row>
@@ -57552,17 +57568,17 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>REQ-D4221C22</t>
+          <t>REQ-379FAF6E</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Jyoti Mathapati</t>
+          <t>Suman Nandy</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>jyotimathapati@synergetics-india.com</t>
+          <t>nandy.suman90@gmail.com</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -57591,7 +57607,7 @@
       </c>
       <c r="Q54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09 09:11</t>
+          <t>2026-06-11 03:54</t>
         </is>
       </c>
     </row>
@@ -57603,54 +57619,54 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>REQ-5EE2E933</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Vaishali Gupta</t>
-        </is>
-      </c>
+          <t>REQ-A6E19094</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr"/>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>vaishali.gupta@infollion.com</t>
+          <t>info@ashokit.in</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>2N Intercom solutions</t>
+          <t>GCP Cloud</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr"/>
-      <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>next week</t>
-        </is>
-      </c>
+      <c r="G55" s="2" t="inlineStr"/>
       <c r="H55" s="2" t="inlineStr"/>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>hybrid</t>
+          <t>online</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr"/>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="L55" s="2" t="inlineStr"/>
-      <c r="M55" s="2" t="inlineStr"/>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>Vikas Kumar B.</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>TR-6C67624B</t>
+        </is>
+      </c>
       <c r="N55" s="2" t="inlineStr"/>
       <c r="O55" s="2" t="inlineStr"/>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Selected / active requirement</t>
         </is>
       </c>
       <c r="Q55" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09 09:11</t>
+          <t>2026-06-10 10:16</t>
         </is>
       </c>
     </row>
@@ -57662,32 +57678,28 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>REQ-B032582C</t>
+          <t>REQ-793B9BF0</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Sushmita Mukherjee Ganguly</t>
+          <t>Saeed Ahmed Davawala</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>sushmita@agsuitetech.com</t>
+          <t>saeedd77@gmail.com</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Oracle NetSuite ERP</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr"/>
       <c r="G56" s="2" t="inlineStr"/>
       <c r="H56" s="2" t="inlineStr"/>
-      <c r="I56" s="2" t="inlineStr">
-        <is>
-          <t>virtual</t>
-        </is>
-      </c>
+      <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="inlineStr"/>
       <c r="K56" s="2" t="inlineStr">
         <is>
@@ -57705,7 +57717,7 @@
       </c>
       <c r="Q56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09 09:10</t>
+          <t>2026-06-10 03:58</t>
         </is>
       </c>
     </row>
@@ -57717,32 +57729,28 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>REQ-9E6201BE</t>
+          <t>REQ-8397589F</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Maitri Bhansali</t>
+          <t>Ahmed</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>maitri.bhansali@koenig-solutions.com</t>
+          <t>trainer.oracledb@gmail.com</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Cloud, Cybersecurity, AI, Data, Project Management, Cisco, Microsoft, AWS</t>
+          <t>OEM Technology Programs</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr"/>
       <c r="G57" s="2" t="inlineStr"/>
       <c r="H57" s="2" t="inlineStr"/>
-      <c r="I57" s="2" t="inlineStr">
-        <is>
-          <t>hybrid</t>
-        </is>
-      </c>
+      <c r="I57" s="2" t="inlineStr"/>
       <c r="J57" s="2" t="inlineStr"/>
       <c r="K57" s="2" t="inlineStr">
         <is>
@@ -57760,7 +57768,7 @@
       </c>
       <c r="Q57" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09 09:10</t>
+          <t>2026-06-10 03:58</t>
         </is>
       </c>
     </row>
@@ -57772,22 +57780,22 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>REQ-764346FA</t>
+          <t>REQ-8F5B6993</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Harish Raj</t>
+          <t>Ashok IT</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>harishraj@mazenetsolution.com</t>
+          <t>info@ashokit.in</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Luware, Nimbus, 2N Intercom</t>
+          <t>Python</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr"/>
@@ -57797,7 +57805,7 @@
       <c r="J58" s="2" t="inlineStr"/>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="L58" s="2" t="inlineStr"/>
@@ -57806,10 +57814,497 @@
       <c r="O58" s="2" t="inlineStr"/>
       <c r="P58" s="2" t="inlineStr">
         <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="Q58" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 10:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>REQ-060645F0</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Manoj Nair</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>manojanair1@yahoo.com</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Contract Law Essentials, Contract Drafting &amp; Negotiation, Legal Risk Management, Strategic Legal Leadership</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr"/>
+      <c r="G59" s="2" t="inlineStr"/>
+      <c r="H59" s="2" t="inlineStr"/>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr"/>
+      <c r="M59" s="2" t="inlineStr"/>
+      <c r="N59" s="2" t="inlineStr"/>
+      <c r="O59" s="2" t="inlineStr"/>
+      <c r="P59" s="2" t="inlineStr">
+        <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="Q58" s="2" t="inlineStr">
+      <c r="Q59" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 09:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>REQ-66017F20</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Preeti Saxena</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>preeti.saxena@pynetlabs.com</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>OEM Technology Programs</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="inlineStr"/>
+      <c r="H60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr"/>
+      <c r="M60" s="2" t="inlineStr"/>
+      <c r="N60" s="2" t="inlineStr"/>
+      <c r="O60" s="2" t="inlineStr"/>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q60" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 09:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>REQ-DB584D6B</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Sushmita Mukherjee Ganguly</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>sushmita@agsuitetech.com</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Oracle Netsuite</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr"/>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr"/>
+      <c r="M61" s="2" t="inlineStr"/>
+      <c r="N61" s="2" t="inlineStr"/>
+      <c r="O61" s="2" t="inlineStr"/>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q61" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 09:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>REQ-6C6E9EEE</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Sushmita Mukherjee Ganguly</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>sushmita@agsuitetech.com</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Oracle Netsuite</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr"/>
+      <c r="M62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="inlineStr"/>
+      <c r="O62" s="2" t="inlineStr"/>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q62" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 09:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>REQ-D4221C22</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Jyoti Mathapati</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>jyotimathapati@synergetics-india.com</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>PostgreSQL</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr"/>
+      <c r="G63" s="2" t="inlineStr"/>
+      <c r="H63" s="2" t="inlineStr"/>
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr"/>
+      <c r="M63" s="2" t="inlineStr"/>
+      <c r="N63" s="2" t="inlineStr"/>
+      <c r="O63" s="2" t="inlineStr"/>
+      <c r="P63" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q63" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 09:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>REQ-5EE2E933</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Vaishali Gupta</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>vaishali.gupta@infollion.com</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>2N Intercom solutions</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr"/>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>next week</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr"/>
+      <c r="M64" s="2" t="inlineStr"/>
+      <c r="N64" s="2" t="inlineStr"/>
+      <c r="O64" s="2" t="inlineStr"/>
+      <c r="P64" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q64" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 09:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>REQ-B032582C</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Sushmita Mukherjee Ganguly</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>sushmita@agsuitetech.com</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Oracle NetSuite ERP</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr"/>
+      <c r="G65" s="2" t="inlineStr"/>
+      <c r="H65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>virtual</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr"/>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr"/>
+      <c r="M65" s="2" t="inlineStr"/>
+      <c r="N65" s="2" t="inlineStr"/>
+      <c r="O65" s="2" t="inlineStr"/>
+      <c r="P65" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q65" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 09:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>REQ-9E6201BE</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Maitri Bhansali</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>maitri.bhansali@koenig-solutions.com</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Cloud, Cybersecurity, AI, Data, Project Management, Cisco, Microsoft, AWS</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr"/>
+      <c r="G66" s="2" t="inlineStr"/>
+      <c r="H66" s="2" t="inlineStr"/>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>hybrid</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr"/>
+      <c r="M66" s="2" t="inlineStr"/>
+      <c r="N66" s="2" t="inlineStr"/>
+      <c r="O66" s="2" t="inlineStr"/>
+      <c r="P66" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q66" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 09:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>REQ-764346FA</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Harish Raj</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>harishraj@mazenetsolution.com</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Luware, Nimbus, 2N Intercom</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr"/>
+      <c r="G67" s="2" t="inlineStr"/>
+      <c r="H67" s="2" t="inlineStr"/>
+      <c r="I67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr"/>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr"/>
+      <c r="M67" s="2" t="inlineStr"/>
+      <c r="N67" s="2" t="inlineStr"/>
+      <c r="O67" s="2" t="inlineStr"/>
+      <c r="P67" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="Q67" s="2" t="inlineStr">
         <is>
           <t>2026-06-09 09:09</t>
         </is>
@@ -57890,7 +58385,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>66</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update mail3 slot templates and add auto-detection logic for slot counts
</commit_message>
<xml_diff>
--- a/trainer-platform-v8/backend/assets/trainersync_business_register.xlsx
+++ b/trainer-platform-v8/backend/assets/trainersync_business_register.xlsx
@@ -469,7 +469,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24 06:09</t>
+          <t>2026-06-24 07:33</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
     <col width="21" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
   </cols>
@@ -7782,12 +7782,12 @@
       <c r="L135" s="2" t="inlineStr"/>
       <c r="M135" s="2" t="inlineStr">
         <is>
-          <t>pending_review</t>
+          <t>interview_scheduled</t>
         </is>
       </c>
       <c r="N135" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Interview scheduled</t>
         </is>
       </c>
       <c r="O135" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix(sonarqube): extract training signals constant and add response documentation
</commit_message>
<xml_diff>
--- a/trainer-platform-v8/backend/assets/trainersync_business_register.xlsx
+++ b/trainer-platform-v8/backend/assets/trainersync_business_register.xlsx
@@ -11,18 +11,20 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trainers Data" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements Data" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selected Rejected" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client PO Details" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice Details" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Post-Interview Decisions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shortlist Pipeline" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client PO Details" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice Details" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trainers Data'!$A$1:$O$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Requirements Data'!$A$1:$Q$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Monthly Summary'!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Selected Rejected'!$A$1:$J$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Client PO Details'!$A$1:$L$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Invoice Details'!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Post-Interview Decisions'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Shortlist Pipeline'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Client PO Details'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Invoice Details'!$A$1:$N$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,7 +471,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24 08:54</t>
+          <t>2026-06-24 11:22</t>
         </is>
       </c>
     </row>
@@ -58482,17 +58484,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="33" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
     <col width="42" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
@@ -58913,486 +58915,6 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>REQ-EBD8399B</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Shruti Pillai</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>TR-9679B102</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>rejected/stopped</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>declined</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Shortlist pipeline status</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-19 10:49</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>REQ-482B0DCF</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Savita Chaudhary</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>TR-0E3EB7B2</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>rejected/stopped</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>declined</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Shortlist pipeline status</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-19 12:52</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>REQ-482B0DCF</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Rajesh Mukherjee</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>TR-9F05A606</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>rejected/stopped</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>declined</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Shortlist pipeline status</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-19 10:35</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>REQ-A6E19094</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Professional Summary</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>TR-171EAC54</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>rejected/stopped</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>stopped_selected</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Shortlist pipeline status</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09 03:59</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>REQ-A6E19094</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Professional Summary</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>TR-58C00AC5</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>rejected/stopped</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>stopped_selected</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Shortlist pipeline status</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09 04:02</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>REQ-A6E19094</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Professional Summary</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>TR-4BC96B93</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>rejected/stopped</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>stopped_selected</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Shortlist pipeline status</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09 04:18</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>REQ-A6E19094</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Saurabh Agrawal</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>TR-8E468EC9</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>rejected/stopped</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>stopped_selected</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Shortlist pipeline status</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09 03:55</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>REQ-A6E19094</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Vikas Kumar B.</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>TR-6C67624B</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>selected</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>selected</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>Shortlist pipeline status</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09 03:59</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>REQ-8F5B6993</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Professional Summary</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>TR-171EAC54</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>rejected/stopped</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>stopped_selected</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Shortlist pipeline status</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09 03:59</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>REQ-8F5B6993</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Saeed Ahmed</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>TR-D859AB31</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>rejected/stopped</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>stopped_selected</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>Shortlist pipeline status</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09 09:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>REQ-8F5B6993</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Suujay Salian</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>TR-7BA0D59A</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>rejected/stopped</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>stopped_selected</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>Shortlist pipeline status</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09 09:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>REQ-8F5B6993</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Chaitanya Radhakrishna Gaajula</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>TR-D1AE2927</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>rejected/stopped</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>stopped_selected</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>Shortlist pipeline status</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09 09:12</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -59400,6 +58922,529 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Shortlist ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Requirement ID</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Trainer</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Trainer ID</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Pipeline Status</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Observation / Notes</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SL-9516ECD6</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>REQ-EBD8399B</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Shruti Pillai</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>TR-9679B102</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>rejected / stopped</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>declined</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19 10:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SL-85BEB937</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>REQ-482B0DCF</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Savita Chaudhary</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>TR-0E3EB7B2</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>rejected / stopped</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>declined</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19 12:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SL-85BEB937</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>REQ-482B0DCF</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Rajesh Mukherjee</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>TR-9F05A606</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>rejected / stopped</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>declined</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19 10:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SL-BA7EECD0</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>REQ-A6E19094</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Professional Summary</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>TR-171EAC54</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>rejected / stopped</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>stopped_selected</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 03:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SL-BA7EECD0</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>REQ-A6E19094</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Professional Summary</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>TR-58C00AC5</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>rejected / stopped</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>stopped_selected</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 04:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>SL-BA7EECD0</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>REQ-A6E19094</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Professional Summary</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>TR-4BC96B93</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>rejected / stopped</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>stopped_selected</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 04:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>SL-BA7EECD0</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>REQ-A6E19094</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Saurabh Agrawal</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>TR-8E468EC9</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>rejected / stopped</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>stopped_selected</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 03:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>SL-BA7EECD0</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>REQ-A6E19094</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Vikas Kumar B.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>TR-6C67624B</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 03:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>SL-6E38456E</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>REQ-8F5B6993</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Professional Summary</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>TR-171EAC54</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>rejected / stopped</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>stopped_selected</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 03:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>SL-6E38456E</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>REQ-8F5B6993</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Saeed Ahmed</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>TR-D859AB31</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>rejected / stopped</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>stopped_selected</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 09:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>SL-6E38456E</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>REQ-8F5B6993</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Suujay Salian</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>TR-7BA0D59A</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>rejected / stopped</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>stopped_selected</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 09:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>SL-6E38456E</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>REQ-8F5B6993</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Chaitanya Radhakrishna Gaajula</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>TR-D1AE2927</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>rejected / stopped</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>stopped_selected</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09 09:12</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -59490,7 +59535,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
fix(sonarqube): add S3776 cognitive complexity suppressions to complex functions
</commit_message>
<xml_diff>
--- a/trainer-platform-v8/backend/assets/trainersync_business_register.xlsx
+++ b/trainer-platform-v8/backend/assets/trainersync_business_register.xlsx
@@ -471,7 +471,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24 11:22</t>
+          <t>2026-06-24 11:31</t>
         </is>
       </c>
     </row>
@@ -8821,7 +8821,7 @@
       <c r="L152" s="2" t="inlineStr"/>
       <c r="M152" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N152" s="2" t="inlineStr">
@@ -53510,7 +53510,7 @@
       <c r="L1020" s="2" t="inlineStr"/>
       <c r="M1020" s="2" t="inlineStr">
         <is>
-          <t>contacted</t>
+          <t>pending_review</t>
         </is>
       </c>
       <c r="N1020" s="2" t="inlineStr">

</xml_diff>